<commit_message>
Remove all JSON report files and enforce EXCEL (.xlsx) files exclusively across repository and GitHub Actions
</commit_message>
<xml_diff>
--- a/app/reports/Mobile_and_Web_App_Test_Report_300_TestCases.xlsx
+++ b/app/reports/Mobile_and_Web_App_Test_Report_300_TestCases.xlsx
@@ -551,9 +551,9 @@
   <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="39" customWidth="1" min="2" max="2"/>
-    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
@@ -572,7 +572,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Run Information &amp; GitHub Actions Artifacts</t>
+          <t>Run Information &amp; GitHub Actions Excel Artifacts</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Artifact SHA256 Digests (GitHub Actions)</t>
+          <t>Excel Artifact Files (.xlsx)</t>
         </is>
       </c>
     </row>
@@ -945,126 +945,126 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>SHA-256 Digest</t>
+          <t>Excel Sheet Name</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>appium-android-report</t>
+          <t>appium-android-report.xlsx</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Excel Sheet (.xlsx)</t>
+          <t>Microsoft Excel (.xlsx)</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>sha256:3a13fa1e6d1dd83c2332726c2a615ec30e35f56c6a9</t>
+          <t>Appium Android Tests</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>selenium-web-report</t>
+          <t>selenium-web-report.xlsx</t>
         </is>
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>Excel Sheet (.xlsx)</t>
+          <t>Microsoft Excel (.xlsx)</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>sha256:29f2b745dea940f4976eca6cbc95fbf44065aae6889</t>
+          <t>Selenium Website Tests</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>unit-test-report</t>
+          <t>unit-test-report.xlsx</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Excel Sheet (.xlsx)</t>
+          <t>Microsoft Excel (.xlsx)</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>sha256:5f5aec0d9c579b78555cb181a23c82ca173072e365d</t>
+          <t>Unit Tests API</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>validation-test-report</t>
+          <t>validation-test-report.xlsx</t>
         </is>
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>Excel Sheet (.xlsx)</t>
+          <t>Microsoft Excel (.xlsx)</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>sha256:ee8b4a0513e4e4b36757c859a23af7c355abeb34dab</t>
+          <t>Validation Tests</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>load-test-report</t>
+          <t>load-test-report.xlsx</t>
         </is>
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>Excel Sheet (.xlsx)</t>
+          <t>Microsoft Excel (.xlsx)</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>sha256:8bb58a1e25c450f1848141b4b07c97c67085a0af097</t>
+          <t>Load Performance Tests</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>deployment-test-report</t>
+          <t>deployment-test-report.xlsx</t>
         </is>
       </c>
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>Excel Sheet (.xlsx)</t>
+          <t>Microsoft Excel (.xlsx)</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>sha256:65c2be0d1b7b50685b4df32a67e2060cb4edc8c83ca</t>
+          <t>Deployment Status</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>full-e2e-report</t>
+          <t>full-e2e-report.xlsx</t>
         </is>
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>Excel Sheet (.xlsx)</t>
+          <t>Microsoft Excel (.xlsx)</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>sha256:ff529cb1597e4e3b8ae597182a1071db63fefbe7ae6</t>
+          <t>Executive Summary + All Suites</t>
         </is>
       </c>
     </row>

</xml_diff>